<commit_message>
Challenge 5 explanation code (number 54)
</commit_message>
<xml_diff>
--- a/Solution explanations.xlsx
+++ b/Solution explanations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ainis\Desktop\LIFE\Coding projects\Daily challanges\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8434753F-F586-48B5-879F-81F65D0ECF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78C21FD8-9C12-43B2-A343-32A04EED45B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BDCE91D3-EC99-46FF-ABB3-2304E474D35E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
   <si>
     <t>Problem name</t>
   </si>
@@ -366,6 +366,12 @@
   </si>
   <si>
     <t>We run binary search, low = 1, high = x,we calculate the middle, raise is to the power of two and check if its equal to x, if we've not found the solution after the while loop has ended we return low - 1</t>
+  </si>
+  <si>
+    <t>Search a 2D Matrix</t>
+  </si>
+  <si>
+    <t>We run binary search, but low = 0 and high = cols * rows - 1, and to get each mid element we get the y = mid // cols and x = mid % cols</t>
   </si>
 </sst>
 </file>
@@ -1978,10 +1984,14 @@
       <c r="B58" s="1">
         <v>54</v>
       </c>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="3"/>
+      <c r="C58" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="3" t="s">
+        <v>110</v>
+      </c>
       <c r="G58" s="3"/>
       <c r="H58" s="3"/>
       <c r="I58" s="3"/>

</xml_diff>